<commit_message>
Editing the excel sheet
</commit_message>
<xml_diff>
--- a/khaledz.xlsx
+++ b/khaledz.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahmedz\github-projects\git_course\git_course\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B40C01-4DFF-4A12-98B1-E2B3E2C2433D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,12 +24,50 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>Column2</t>
+  </si>
+  <si>
+    <t>Column3</t>
+  </si>
+  <si>
+    <t>Column4</t>
+  </si>
+  <si>
+    <t>Column5</t>
+  </si>
+  <si>
+    <t>Column6</t>
+  </si>
+  <si>
+    <t>Column7</t>
+  </si>
+  <si>
+    <t>Column8</t>
+  </si>
+  <si>
+    <t>Column9</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -66,6 +110,21 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9EC2080B-4520-4A5B-BEF9-93F37C82426F}" name="Table1" displayName="Table1" ref="A1:F2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:F2" xr:uid="{9EC2080B-4520-4A5B-BEF9-93F37C82426F}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{2CFB1FD3-E961-4FF8-A8C5-24CB27AD480D}" name="Column1"/>
+    <tableColumn id="2" xr3:uid="{66794D31-4E0D-4470-876C-58D712728110}" name="Column2"/>
+    <tableColumn id="3" xr3:uid="{14FA8BA2-C3A0-4DC9-8CB4-31D33375CD62}" name="Column3"/>
+    <tableColumn id="4" xr3:uid="{7EA0E8AE-BC5A-4855-9DBC-99E7AF8B82F1}" name="Column4"/>
+    <tableColumn id="5" xr3:uid="{40989C23-389E-48DB-96BA-546C58B448A0}" name="Column5"/>
+    <tableColumn id="6" xr3:uid="{38B86B2C-79D7-425E-8635-3B0A0FDEB3E0}" name="Column6"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -330,10 +389,78 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>